<commit_message>
update cop lagi- ke 6
</commit_message>
<xml_diff>
--- a/template_pst.xlsx
+++ b/template_pst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\#Project_Web\Website_E-Perjadin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF10F27D-C29D-4A9C-8181-DEE040F3E472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E7A647-72FA-41F2-B1DE-1E79E559DFA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{90350066-7765-4977-A66B-164B7EBDC2B4}"/>
   </bookViews>
@@ -1695,6 +1695,171 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1709,171 +1874,6 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1899,15 +1899,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>228985</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>259963</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>4130</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1922,28 +1922,25 @@
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect l="30870" t="19362" r="30664" b="69631"/>
+        <a:srcRect/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="8866481" cy="1440089"/>
+          <a:off x="228985" y="0"/>
+          <a:ext cx="8675447" cy="1432880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
         <a:extLst>
           <a:ext uri="{53640926-AAD7-44D8-BBD7-CCE9431645EC}">
             <a14:shadowObscured xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main"/>
@@ -1961,22 +1958,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>24262</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>253863</xdr:colOff>
+      <xdr:colOff>234699</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>69273</xdr:rowOff>
+      <xdr:rowOff>92364</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5FABC2E7-2D1A-4959-7A18-FE58AB4FC60E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{692EE0FA-F083-4412-903B-C1014FE1CC57}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1984,28 +1981,25 @@
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect l="30870" t="19362" r="30664" b="69631"/>
+        <a:srcRect/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="24262" y="0"/>
-          <a:ext cx="8103601" cy="1316182"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="8108699" cy="1339273"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
         <a:extLst>
           <a:ext uri="{53640926-AAD7-44D8-BBD7-CCE9431645EC}">
             <a14:shadowObscured xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main"/>
@@ -2294,96 +2288,96 @@
   <sheetData>
     <row r="1" spans="1:9" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B1" s="1"/>
-      <c r="C1" s="155"/>
-      <c r="D1" s="155"/>
-      <c r="E1" s="155"/>
-      <c r="F1" s="155"/>
-      <c r="G1" s="155"/>
+      <c r="C1" s="148"/>
+      <c r="D1" s="148"/>
+      <c r="E1" s="148"/>
+      <c r="F1" s="148"/>
+      <c r="G1" s="148"/>
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="2"/>
-      <c r="C2" s="155"/>
-      <c r="D2" s="155"/>
-      <c r="E2" s="155"/>
-      <c r="F2" s="155"/>
-      <c r="G2" s="155"/>
+      <c r="C2" s="148"/>
+      <c r="D2" s="148"/>
+      <c r="E2" s="148"/>
+      <c r="F2" s="148"/>
+      <c r="G2" s="148"/>
       <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:9" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3"/>
-      <c r="C3" s="156"/>
-      <c r="D3" s="156"/>
-      <c r="E3" s="156"/>
-      <c r="F3" s="156"/>
-      <c r="G3" s="156"/>
+      <c r="C3" s="149"/>
+      <c r="D3" s="149"/>
+      <c r="E3" s="149"/>
+      <c r="F3" s="149"/>
+      <c r="G3" s="149"/>
       <c r="H3" s="3"/>
     </row>
     <row r="4" spans="1:9" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4"/>
-      <c r="C4" s="157"/>
-      <c r="D4" s="157"/>
-      <c r="E4" s="157"/>
-      <c r="F4" s="157"/>
-      <c r="G4" s="157"/>
+      <c r="C4" s="150"/>
+      <c r="D4" s="150"/>
+      <c r="E4" s="150"/>
+      <c r="F4" s="150"/>
+      <c r="G4" s="150"/>
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B5" s="5"/>
-      <c r="C5" s="158"/>
-      <c r="D5" s="158"/>
-      <c r="E5" s="158"/>
-      <c r="F5" s="158"/>
-      <c r="G5" s="158"/>
+      <c r="C5" s="151"/>
+      <c r="D5" s="151"/>
+      <c r="E5" s="151"/>
+      <c r="F5" s="151"/>
+      <c r="G5" s="151"/>
       <c r="H5" s="5"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B6" s="6"/>
-      <c r="C6" s="159"/>
-      <c r="D6" s="159"/>
-      <c r="E6" s="159"/>
-      <c r="F6" s="159"/>
-      <c r="G6" s="159"/>
+      <c r="C6" s="152"/>
+      <c r="D6" s="152"/>
+      <c r="E6" s="152"/>
+      <c r="F6" s="152"/>
+      <c r="G6" s="152"/>
       <c r="H6" s="6"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="F7" s="7"/>
     </row>
     <row r="9" spans="1:9" ht="22.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="154" t="s">
+      <c r="A9" s="147" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="154"/>
-      <c r="C9" s="154"/>
-      <c r="D9" s="154"/>
-      <c r="E9" s="154"/>
-      <c r="F9" s="154"/>
-      <c r="G9" s="154"/>
+      <c r="B9" s="147"/>
+      <c r="C9" s="147"/>
+      <c r="D9" s="147"/>
+      <c r="E9" s="147"/>
+      <c r="F9" s="147"/>
+      <c r="G9" s="147"/>
       <c r="H9" s="8"/>
     </row>
     <row r="10" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="160" t="s">
+      <c r="A10" s="138" t="s">
         <v>101</v>
       </c>
-      <c r="B10" s="160"/>
-      <c r="C10" s="160"/>
-      <c r="D10" s="160"/>
-      <c r="E10" s="160"/>
-      <c r="F10" s="160"/>
-      <c r="G10" s="160"/>
+      <c r="B10" s="138"/>
+      <c r="C10" s="138"/>
+      <c r="D10" s="138"/>
+      <c r="E10" s="138"/>
+      <c r="F10" s="138"/>
+      <c r="G10" s="138"/>
       <c r="H10" s="10"/>
       <c r="I10" s="39"/>
     </row>
     <row r="11" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="160" t="s">
+      <c r="A11" s="138" t="s">
         <v>106</v>
       </c>
-      <c r="B11" s="160"/>
-      <c r="C11" s="160"/>
-      <c r="D11" s="160"/>
-      <c r="E11" s="160"/>
-      <c r="F11" s="160"/>
-      <c r="G11" s="160"/>
+      <c r="B11" s="138"/>
+      <c r="C11" s="138"/>
+      <c r="D11" s="138"/>
+      <c r="E11" s="138"/>
+      <c r="F11" s="138"/>
+      <c r="G11" s="138"/>
       <c r="H11" s="10"/>
       <c r="I11" s="39"/>
     </row>
@@ -2473,11 +2467,11 @@
       <c r="D17" s="128" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="161" t="s">
+      <c r="E17" s="139" t="s">
         <v>63</v>
       </c>
-      <c r="F17" s="162"/>
-      <c r="G17" s="162"/>
+      <c r="F17" s="140"/>
+      <c r="G17" s="140"/>
       <c r="H17" s="14"/>
     </row>
     <row r="18" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
@@ -2520,11 +2514,11 @@
       <c r="C21" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="D21" s="163" t="s">
+      <c r="D21" s="141" t="s">
         <v>67</v>
       </c>
-      <c r="E21" s="164"/>
-      <c r="F21" s="165"/>
+      <c r="E21" s="142"/>
+      <c r="F21" s="143"/>
       <c r="G21" s="19" t="s">
         <v>30</v>
       </c>
@@ -2539,12 +2533,12 @@
         <f>'Permohonan Perjadin'!C15</f>
         <v>Dr. Ir. I Ketut Kariyasa, M.Si.</v>
       </c>
-      <c r="D22" s="166" t="str">
+      <c r="D22" s="144" t="str">
         <f>'Permohonan Perjadin'!I15</f>
         <v>IV/d</v>
       </c>
-      <c r="E22" s="167"/>
-      <c r="F22" s="168"/>
+      <c r="E22" s="145"/>
+      <c r="F22" s="146"/>
       <c r="G22" s="131" t="str">
         <f>'Permohonan Perjadin'!F15</f>
         <v>Kepala Pusat</v>
@@ -2560,12 +2554,12 @@
         <f>'Permohonan Perjadin'!C16</f>
         <v>Hamdan Mubarok</v>
       </c>
-      <c r="D23" s="169" t="str">
+      <c r="D23" s="135" t="str">
         <f>'Permohonan Perjadin'!I16</f>
         <v>V</v>
       </c>
-      <c r="E23" s="170"/>
-      <c r="F23" s="171"/>
+      <c r="E23" s="136"/>
+      <c r="F23" s="137"/>
       <c r="G23" s="132" t="str">
         <f>'Permohonan Perjadin'!F16</f>
         <v>Pengadministrasi Perkantoran</v>
@@ -2576,9 +2570,9 @@
       <c r="A24" s="21"/>
       <c r="B24" s="25"/>
       <c r="C24" s="23"/>
-      <c r="D24" s="169"/>
-      <c r="E24" s="170"/>
-      <c r="F24" s="171"/>
+      <c r="D24" s="135"/>
+      <c r="E24" s="136"/>
+      <c r="F24" s="137"/>
       <c r="G24" s="132"/>
       <c r="H24" s="24"/>
     </row>
@@ -2586,9 +2580,9 @@
       <c r="A25" s="21"/>
       <c r="B25" s="25"/>
       <c r="C25" s="23"/>
-      <c r="D25" s="169"/>
-      <c r="E25" s="170"/>
-      <c r="F25" s="171"/>
+      <c r="D25" s="135"/>
+      <c r="E25" s="136"/>
+      <c r="F25" s="137"/>
       <c r="G25" s="132"/>
       <c r="H25" s="24"/>
     </row>
@@ -2864,6 +2858,13 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="C1:G1"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="C6:G6"/>
     <mergeCell ref="D25:F25"/>
     <mergeCell ref="D24:F24"/>
     <mergeCell ref="D23:F23"/>
@@ -2872,13 +2873,6 @@
     <mergeCell ref="E17:G17"/>
     <mergeCell ref="D21:F21"/>
     <mergeCell ref="D22:F22"/>
-    <mergeCell ref="A9:G9"/>
-    <mergeCell ref="C1:G1"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="C6:G6"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.19685039370078741" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="77" orientation="portrait" r:id="rId1"/>
@@ -2909,62 +2903,62 @@
       <c r="H1"/>
     </row>
     <row r="2" spans="1:12" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="C2" s="179"/>
-      <c r="D2" s="179"/>
-      <c r="E2" s="179"/>
-      <c r="F2" s="179"/>
-      <c r="G2" s="179"/>
-      <c r="H2" s="179"/>
-      <c r="I2" s="179"/>
+      <c r="C2" s="172"/>
+      <c r="D2" s="172"/>
+      <c r="E2" s="172"/>
+      <c r="F2" s="172"/>
+      <c r="G2" s="172"/>
+      <c r="H2" s="172"/>
+      <c r="I2" s="172"/>
     </row>
     <row r="3" spans="1:12" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="C3" s="155"/>
-      <c r="D3" s="155"/>
-      <c r="E3" s="155"/>
-      <c r="F3" s="155"/>
-      <c r="G3" s="155"/>
-      <c r="H3" s="155"/>
-      <c r="I3" s="155"/>
+      <c r="C3" s="148"/>
+      <c r="D3" s="148"/>
+      <c r="E3" s="148"/>
+      <c r="F3" s="148"/>
+      <c r="G3" s="148"/>
+      <c r="H3" s="148"/>
+      <c r="I3" s="148"/>
       <c r="J3" s="62"/>
       <c r="L3" s="62"/>
     </row>
     <row r="4" spans="1:12" ht="18" x14ac:dyDescent="0.35">
-      <c r="C4" s="180"/>
-      <c r="D4" s="180"/>
-      <c r="E4" s="180"/>
-      <c r="F4" s="180"/>
-      <c r="G4" s="180"/>
-      <c r="H4" s="180"/>
-      <c r="I4" s="180"/>
+      <c r="C4" s="173"/>
+      <c r="D4" s="173"/>
+      <c r="E4" s="173"/>
+      <c r="F4" s="173"/>
+      <c r="G4" s="173"/>
+      <c r="H4" s="173"/>
+      <c r="I4" s="173"/>
       <c r="J4" s="2"/>
       <c r="L4" s="2"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="C5" s="181"/>
-      <c r="D5" s="181"/>
-      <c r="E5" s="181"/>
-      <c r="F5" s="181"/>
-      <c r="G5" s="181"/>
-      <c r="H5" s="181"/>
-      <c r="I5" s="181"/>
+      <c r="C5" s="174"/>
+      <c r="D5" s="174"/>
+      <c r="E5" s="174"/>
+      <c r="F5" s="174"/>
+      <c r="G5" s="174"/>
+      <c r="H5" s="174"/>
+      <c r="I5" s="174"/>
     </row>
     <row r="6" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C6" s="182"/>
-      <c r="D6" s="182"/>
-      <c r="E6" s="182"/>
-      <c r="F6" s="182"/>
-      <c r="G6" s="182"/>
-      <c r="H6" s="182"/>
-      <c r="I6" s="182"/>
+      <c r="C6" s="175"/>
+      <c r="D6" s="175"/>
+      <c r="E6" s="175"/>
+      <c r="F6" s="175"/>
+      <c r="G6" s="175"/>
+      <c r="H6" s="175"/>
+      <c r="I6" s="175"/>
     </row>
     <row r="7" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C7" s="172"/>
-      <c r="D7" s="172"/>
-      <c r="E7" s="172"/>
-      <c r="F7" s="172"/>
-      <c r="G7" s="172"/>
-      <c r="H7" s="172"/>
-      <c r="I7" s="172"/>
+      <c r="C7" s="169"/>
+      <c r="D7" s="169"/>
+      <c r="E7" s="169"/>
+      <c r="F7" s="169"/>
+      <c r="G7" s="169"/>
+      <c r="H7" s="169"/>
+      <c r="I7" s="169"/>
       <c r="J7" s="63"/>
       <c r="L7" s="63"/>
     </row>
@@ -3008,32 +3002,32 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="43"/>
-      <c r="B13" s="189" t="s">
+      <c r="B13" s="161" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="173" t="s">
+      <c r="C13" s="170" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="174"/>
+      <c r="D13" s="167"/>
       <c r="E13" s="44"/>
-      <c r="F13" s="173" t="s">
+      <c r="F13" s="170" t="s">
         <v>30</v>
       </c>
-      <c r="G13" s="174"/>
-      <c r="H13" s="175"/>
+      <c r="G13" s="167"/>
+      <c r="H13" s="171"/>
       <c r="I13" s="64" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" s="43"/>
-      <c r="B14" s="190"/>
-      <c r="C14" s="176"/>
-      <c r="D14" s="177"/>
+      <c r="B14" s="162"/>
+      <c r="C14" s="155"/>
+      <c r="D14" s="168"/>
       <c r="E14" s="45"/>
-      <c r="F14" s="176"/>
-      <c r="G14" s="177"/>
-      <c r="H14" s="178"/>
+      <c r="F14" s="155"/>
+      <c r="G14" s="168"/>
+      <c r="H14" s="156"/>
       <c r="I14" s="65" t="s">
         <v>32</v>
       </c>
@@ -3048,11 +3042,11 @@
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="12"/>
-      <c r="F15" s="191" t="s">
+      <c r="F15" s="163" t="s">
         <v>87</v>
       </c>
-      <c r="G15" s="192"/>
-      <c r="H15" s="193"/>
+      <c r="G15" s="164"/>
+      <c r="H15" s="165"/>
       <c r="I15" s="66" t="s">
         <v>88</v>
       </c>
@@ -3067,11 +3061,11 @@
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="12"/>
-      <c r="F16" s="191" t="s">
+      <c r="F16" s="163" t="s">
         <v>91</v>
       </c>
-      <c r="G16" s="192"/>
-      <c r="H16" s="193"/>
+      <c r="G16" s="164"/>
+      <c r="H16" s="165"/>
       <c r="I16" s="66" t="s">
         <v>83</v>
       </c>
@@ -3082,9 +3076,9 @@
       <c r="C17" s="15"/>
       <c r="D17" s="12"/>
       <c r="E17" s="12"/>
-      <c r="F17" s="191"/>
-      <c r="G17" s="192"/>
-      <c r="H17" s="193"/>
+      <c r="F17" s="163"/>
+      <c r="G17" s="164"/>
+      <c r="H17" s="165"/>
       <c r="I17" s="66"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
@@ -3093,9 +3087,9 @@
       <c r="C18" s="15"/>
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
-      <c r="F18" s="191"/>
-      <c r="G18" s="192"/>
-      <c r="H18" s="193"/>
+      <c r="F18" s="163"/>
+      <c r="G18" s="164"/>
+      <c r="H18" s="165"/>
       <c r="I18" s="66"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
@@ -3197,10 +3191,10 @@
       <c r="D26" s="129" t="s">
         <v>36</v>
       </c>
-      <c r="E26" s="194" t="s">
+      <c r="E26" s="166" t="s">
         <v>104</v>
       </c>
-      <c r="F26" s="192"/>
+      <c r="F26" s="164"/>
       <c r="G26" s="118" t="s">
         <v>98</v>
       </c>
@@ -3217,10 +3211,10 @@
       <c r="D27" s="129" t="s">
         <v>36</v>
       </c>
-      <c r="E27" s="194" t="s">
+      <c r="E27" s="166" t="s">
         <v>84</v>
       </c>
-      <c r="F27" s="192"/>
+      <c r="F27" s="164"/>
       <c r="G27" s="26"/>
       <c r="H27" s="26"/>
     </row>
@@ -3496,24 +3490,24 @@
     </row>
     <row r="50" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="12"/>
-      <c r="B50" s="183" t="s">
+      <c r="B50" s="153" t="s">
         <v>53</v>
       </c>
-      <c r="C50" s="184"/>
-      <c r="D50" s="185" t="s">
+      <c r="C50" s="154"/>
+      <c r="D50" s="157" t="s">
         <v>54</v>
       </c>
-      <c r="E50" s="186"/>
+      <c r="E50" s="158"/>
       <c r="F50" s="41"/>
       <c r="G50" s="12"/>
       <c r="H50" s="12"/>
     </row>
     <row r="51" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="12"/>
-      <c r="B51" s="176"/>
-      <c r="C51" s="178"/>
-      <c r="D51" s="187"/>
-      <c r="E51" s="188"/>
+      <c r="B51" s="155"/>
+      <c r="C51" s="156"/>
+      <c r="D51" s="159"/>
+      <c r="E51" s="160"/>
       <c r="F51" s="41"/>
       <c r="G51" s="12"/>
       <c r="H51" s="12"/>
@@ -3714,6 +3708,14 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="F13:H14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="C2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
     <mergeCell ref="B50:C51"/>
     <mergeCell ref="D50:E51"/>
     <mergeCell ref="B13:B14"/>
@@ -3724,14 +3726,6 @@
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="F18:H18"/>
     <mergeCell ref="F17:H17"/>
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="F13:H14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="C6:I6"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.19685039370078741" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="82" orientation="portrait" r:id="rId1"/>
@@ -3765,62 +3759,62 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A2" s="135" t="s">
+      <c r="A2" s="190" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="135"/>
-      <c r="C2" s="135"/>
-      <c r="D2" s="135"/>
-      <c r="E2" s="135"/>
-      <c r="F2" s="135"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="135"/>
-      <c r="I2" s="135"/>
-      <c r="J2" s="135"/>
-      <c r="K2" s="135"/>
-      <c r="L2" s="135"/>
-      <c r="M2" s="135"/>
-      <c r="N2" s="135"/>
-      <c r="O2" s="135"/>
-      <c r="P2" s="135"/>
+      <c r="B2" s="190"/>
+      <c r="C2" s="190"/>
+      <c r="D2" s="190"/>
+      <c r="E2" s="190"/>
+      <c r="F2" s="190"/>
+      <c r="G2" s="190"/>
+      <c r="H2" s="190"/>
+      <c r="I2" s="190"/>
+      <c r="J2" s="190"/>
+      <c r="K2" s="190"/>
+      <c r="L2" s="190"/>
+      <c r="M2" s="190"/>
+      <c r="N2" s="190"/>
+      <c r="O2" s="190"/>
+      <c r="P2" s="190"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A3" s="135" t="s">
+      <c r="A3" s="190" t="s">
         <v>97</v>
       </c>
-      <c r="B3" s="135"/>
-      <c r="C3" s="135"/>
-      <c r="D3" s="135"/>
-      <c r="E3" s="135"/>
-      <c r="F3" s="135"/>
-      <c r="G3" s="135"/>
-      <c r="H3" s="135"/>
-      <c r="I3" s="135"/>
-      <c r="J3" s="135"/>
-      <c r="K3" s="135"/>
-      <c r="L3" s="135"/>
-      <c r="M3" s="135"/>
-      <c r="N3" s="135"/>
-      <c r="O3" s="135"/>
-      <c r="P3" s="135"/>
+      <c r="B3" s="190"/>
+      <c r="C3" s="190"/>
+      <c r="D3" s="190"/>
+      <c r="E3" s="190"/>
+      <c r="F3" s="190"/>
+      <c r="G3" s="190"/>
+      <c r="H3" s="190"/>
+      <c r="I3" s="190"/>
+      <c r="J3" s="190"/>
+      <c r="K3" s="190"/>
+      <c r="L3" s="190"/>
+      <c r="M3" s="190"/>
+      <c r="N3" s="190"/>
+      <c r="O3" s="190"/>
+      <c r="P3" s="190"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A4" s="136"/>
-      <c r="B4" s="136"/>
-      <c r="C4" s="136"/>
-      <c r="D4" s="136"/>
-      <c r="E4" s="136"/>
-      <c r="F4" s="136"/>
-      <c r="G4" s="136"/>
-      <c r="H4" s="136"/>
-      <c r="I4" s="136"/>
-      <c r="J4" s="136"/>
-      <c r="K4" s="136"/>
-      <c r="L4" s="136"/>
-      <c r="M4" s="136"/>
-      <c r="N4" s="136"/>
-      <c r="O4" s="136"/>
-      <c r="P4" s="136"/>
+      <c r="A4" s="191"/>
+      <c r="B4" s="191"/>
+      <c r="C4" s="191"/>
+      <c r="D4" s="191"/>
+      <c r="E4" s="191"/>
+      <c r="F4" s="191"/>
+      <c r="G4" s="191"/>
+      <c r="H4" s="191"/>
+      <c r="I4" s="191"/>
+      <c r="J4" s="191"/>
+      <c r="K4" s="191"/>
+      <c r="L4" s="191"/>
+      <c r="M4" s="191"/>
+      <c r="N4" s="191"/>
+      <c r="O4" s="191"/>
+      <c r="P4" s="191"/>
     </row>
     <row r="5" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="39"/>
@@ -3864,16 +3858,16 @@
       <c r="P6" s="39"/>
     </row>
     <row r="7" spans="1:17" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="142" t="s">
+      <c r="A7" s="178" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="144" t="s">
+      <c r="B7" s="180" t="s">
         <v>3</v>
       </c>
       <c r="C7" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="144" t="s">
+      <c r="D7" s="180" t="s">
         <v>5</v>
       </c>
       <c r="E7" s="70" t="s">
@@ -3882,60 +3876,60 @@
       <c r="F7" s="70" t="s">
         <v>7</v>
       </c>
-      <c r="G7" s="137" t="s">
+      <c r="G7" s="192" t="s">
         <v>8</v>
       </c>
-      <c r="H7" s="137"/>
-      <c r="I7" s="146" t="s">
+      <c r="H7" s="192"/>
+      <c r="I7" s="182" t="s">
         <v>9</v>
       </c>
-      <c r="J7" s="146" t="s">
+      <c r="J7" s="182" t="s">
         <v>10</v>
       </c>
       <c r="K7" s="113" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="149" t="s">
+      <c r="L7" s="185" t="s">
         <v>12</v>
       </c>
-      <c r="M7" s="149" t="s">
+      <c r="M7" s="185" t="s">
         <v>13</v>
       </c>
       <c r="N7" s="70"/>
       <c r="O7" s="115" t="s">
         <v>14</v>
       </c>
-      <c r="P7" s="152" t="s">
+      <c r="P7" s="188" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="20.149999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="143"/>
-      <c r="B8" s="145"/>
+      <c r="A8" s="179"/>
+      <c r="B8" s="181"/>
       <c r="C8" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="145"/>
+      <c r="D8" s="181"/>
       <c r="E8" s="71" t="s">
         <v>17</v>
       </c>
       <c r="F8" s="71" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="138" t="s">
+      <c r="G8" s="193" t="s">
         <v>19</v>
       </c>
-      <c r="H8" s="139"/>
-      <c r="I8" s="147"/>
-      <c r="J8" s="148"/>
+      <c r="H8" s="194"/>
+      <c r="I8" s="183"/>
+      <c r="J8" s="184"/>
       <c r="K8" s="114"/>
-      <c r="L8" s="150"/>
-      <c r="M8" s="151"/>
+      <c r="L8" s="186"/>
+      <c r="M8" s="187"/>
       <c r="N8" s="71"/>
       <c r="O8" s="116" t="s">
         <v>20</v>
       </c>
-      <c r="P8" s="153"/>
+      <c r="P8" s="189"/>
     </row>
     <row r="9" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A9" s="72">
@@ -4315,12 +4309,12 @@
       <c r="K23" s="39"/>
       <c r="L23" s="39"/>
       <c r="M23" s="39"/>
-      <c r="N23" s="140" t="str">
+      <c r="N23" s="176" t="str">
         <f>'Permohonan Perjadin'!H35</f>
         <v>Dr. Ir. I Ketut Kariyasa, M.Si</v>
       </c>
-      <c r="O23" s="140"/>
-      <c r="P23" s="140"/>
+      <c r="O23" s="176"/>
+      <c r="P23" s="176"/>
       <c r="R23" s="107"/>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.35">
@@ -4340,12 +4334,12 @@
       <c r="K24" s="39"/>
       <c r="L24" s="39"/>
       <c r="M24" s="39"/>
-      <c r="N24" s="141" t="str">
+      <c r="N24" s="177" t="str">
         <f>'Permohonan Perjadin'!H36</f>
         <v>NIP. 196904191998031002</v>
       </c>
-      <c r="O24" s="141"/>
-      <c r="P24" s="141"/>
+      <c r="O24" s="177"/>
+      <c r="P24" s="177"/>
       <c r="R24" s="107"/>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.35">
@@ -4368,6 +4362,11 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A4:P4"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
     <mergeCell ref="N23:P23"/>
     <mergeCell ref="N24:P24"/>
     <mergeCell ref="A7:A8"/>
@@ -4378,11 +4377,6 @@
     <mergeCell ref="L7:L8"/>
     <mergeCell ref="M7:M8"/>
     <mergeCell ref="P7:P8"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="A3:P3"/>
-    <mergeCell ref="A4:P4"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
   </mergeCells>
   <phoneticPr fontId="23" type="noConversion"/>
   <pageMargins left="0.55118110236220474" right="3.937007874015748E-2" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>